<commit_message>
feat: complete PRD-079 plan trial quota types
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5221,7 +5221,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-14。PRD-078 已完成；PRD-079 仅完成权威范围交叉确认，尚未实现。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-14。PRD-079 已完成；PRD-080 已完成权威范围交叉确认但未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="G6" s="46" t="inlineStr">
         <is>
-          <t>未开始（下一项，仅交叉确认）</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="H6" s="45" t="inlineStr">
@@ -5423,27 +5423,27 @@
       </c>
       <c r="I6" s="45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>72/0072 -&gt; 72/0072 -&gt; 71/0071 -&gt; 72/0072；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J6" s="45" t="inlineStr">
         <is>
-          <t>未执行</t>
+          <t>PRD-079 Python 73；Console 792/792；Browser 合同 9/9；OpenAI 28；FinOps/Webhook 26；兼容回归 29</t>
         </is>
       </c>
       <c r="K6" s="45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>.artifacts/prd079-runtime/run-agent4-b72e1d</t>
         </is>
       </c>
       <c r="L6" s="45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>.artifacts/prd079-browser/main-browser-final-20260814-i</t>
         </is>
       </c>
       <c r="M6" s="45" t="inlineStr">
         <is>
-          <t>01_PRD总表第80行；03_M2-M3扩展交付第16行；PAGE-110/111；TC-0157/0158</t>
+          <t>docs/prd/PRD-079-plan-trial-quota-types.md；docs/api/plan-billing.md；docs/testing/PRD-079-tests.md</t>
         </is>
       </c>
       <c r="N6" s="45" t="b">
@@ -5453,7 +5453,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="47" t="inlineStr">
         <is>
-          <t>PRD-078 权威证据摘要</t>
+          <t>PRD-079 权威证据摘要</t>
         </is>
       </c>
       <c r="B8" s="1" t="n"/>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>5a3930e775654a3503241a464e37b206d3850db50c45c7b58b5f7fcf5cb43411</t>
+          <t>c09609cb3e03941721a4ea4e8c023136b543cec57b8d5efd9aa3ea649ec5ae5d</t>
         </is>
       </c>
       <c r="C9" s="52" t="n"/>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="B10" s="51" t="inlineStr">
         <is>
-          <t>49ca9259490a12663cfbad3d441a4dc90a8a103f98ad5067f20616b20d4b5713</t>
+          <t>82a5e2b63dbc0f4aefc9c38cd5bf74e25663643a278b0aeeda4c2c4fe57e72cd</t>
         </is>
       </c>
       <c r="C10" s="52" t="n"/>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="B11" s="49" t="inlineStr">
         <is>
-          <t>600dad48b961ecde342f378776ded8c92fe8bfb83cef12c92bc0c758a33c3065</t>
+          <t>94c6a74fb0a223f07e7a035576d46dc1ef31d3be3c3755bba5e8a59b811705a7</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="B12" s="51" t="inlineStr">
         <is>
-          <t>两轮编码前自审和两轮实现后自审均已完成并修正；无未关闭 P0/P1。</t>
+          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终安全与范围复核无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="B13" s="49" t="inlineStr">
         <is>
-          <t>Excel 总表第80行、M2/M3第16行、PAGE-110/111、Plan/QuotaBucket、quota.exhausted/trial.expired、TC-0157/0158 共同确认 PRD-079；本次未实现。</t>
+          <t>Excel 总表第81行、M2/M3第17行、PAGE-112、BillingDispute/AdjustmentRecord、billing_dispute.created、TC-0159/0160 共同确认 PRD-080；本次未实现。</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>

</xml_diff>

<commit_message>
feat: complete PRD-080 billing dispute adjustment workflow
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5221,7 +5221,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-14。PRD-079 已完成；PRD-080 已完成权威范围交叉确认但未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-15。PRD-080 已完成；下一条权威未完成项为 PRD-081，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -5450,10 +5450,80 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="45" t="inlineStr">
+        <is>
+          <t>PRD-080</t>
+        </is>
+      </c>
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>M2-企业增强</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t>扩展层</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>账单争议</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>账单争议与调整流程</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H7" s="45" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="I7" s="45" t="inlineStr">
+        <is>
+          <t>73/0073 -&gt; 73/0073 -&gt; 72/0072 -&gt; 73/0073；四阶段 integrity=ok、FK=0</t>
+        </is>
+      </c>
+      <c r="J7" s="45" t="inlineStr">
+        <is>
+          <t>PRD-080 Python 58 passed；Console 815/815；Browser 合同 13/13；PRD-078/079 当前链 30 passed</t>
+        </is>
+      </c>
+      <c r="K7" s="45" t="inlineStr">
+        <is>
+          <t>.artifacts/prd080-runtime/prd080-runtime-final-20260815-05</t>
+        </is>
+      </c>
+      <c r="L7" s="45" t="inlineStr">
+        <is>
+          <t>.artifacts/prd080-browser/prd080-browser-final-20260815-05</t>
+        </is>
+      </c>
+      <c r="M7" s="45" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-080-billing-dispute-adjustment-workflow.md；docs/api/billing-disputes.md；docs/testing/PRD-080-tests.md</t>
+        </is>
+      </c>
+      <c r="N7" s="45" t="b">
+        <v>0</v>
+      </c>
+    </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="47" t="inlineStr">
         <is>
-          <t>PRD-079 权威证据摘要</t>
+          <t>PRD-080 权威证据摘要</t>
         </is>
       </c>
       <c r="B8" s="1" t="n"/>
@@ -5478,7 +5548,7 @@
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>c09609cb3e03941721a4ea4e8c023136b543cec57b8d5efd9aa3ea649ec5ae5d</t>
+          <t>74174e1a88553644e08a9584e54e1e866206b943873630c86ecf09fe7619bfd7</t>
         </is>
       </c>
       <c r="C9" s="52" t="n"/>
@@ -5502,7 +5572,7 @@
       </c>
       <c r="B10" s="51" t="inlineStr">
         <is>
-          <t>82a5e2b63dbc0f4aefc9c38cd5bf74e25663643a278b0aeeda4c2c4fe57e72cd</t>
+          <t>a119250da461f04e966c3867f017084d6048eaf53d56877a0fcfef2a653e5193</t>
         </is>
       </c>
       <c r="C10" s="52" t="n"/>
@@ -5526,7 +5596,7 @@
       </c>
       <c r="B11" s="49" t="inlineStr">
         <is>
-          <t>94c6a74fb0a223f07e7a035576d46dc1ef31d3be3c3755bba5e8a59b811705a7</t>
+          <t>c0d53161ee0c1463c1cd98cd07d0fa58cd18f8a92b62faf42e71d2935bb12a99</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>
@@ -5550,7 +5620,7 @@
       </c>
       <c r="B12" s="51" t="inlineStr">
         <is>
-          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终安全与范围复核无未关闭 P0/P1。</t>
+          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终隐私、错误边界、金额聚合复核无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>
@@ -5574,7 +5644,7 @@
       </c>
       <c r="B13" s="49" t="inlineStr">
         <is>
-          <t>Excel 总表第81行、M2/M3第17行、PAGE-112、BillingDispute/AdjustmentRecord、billing_dispute.created、TC-0159/0160 共同确认 PRD-080；本次未实现。</t>
+          <t>Excel 总表第82行、M2/M3第18行、PAGE-113、Webhook format API、SecurityEventPayload、security.event_pushed、TC-0161/0162 共同确认 PRD-081；本次未实现。</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>

</xml_diff>

<commit_message>
feat: complete PRD-081 SIEM security event format
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5221,7 +5221,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-15。PRD-080 已完成；下一条权威未完成项为 PRD-081，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-16。PRD-081 已完成；下一条权威未完成项为 PRD-082，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -5313,7 +5313,7 @@
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="43" t="inlineStr">
         <is>
-          <t>PRD-078</t>
+          <t>PRD-079</t>
         </is>
       </c>
       <c r="B5" s="43" t="inlineStr">
@@ -5333,12 +5333,12 @@
       </c>
       <c r="E5" s="43" t="inlineStr">
         <is>
-          <t>移动审批</t>
+          <t>套餐计费</t>
         </is>
       </c>
       <c r="F5" s="43" t="inlineStr">
         <is>
-          <t>移动端/企微钉钉审批入口</t>
+          <t>套餐、试用与额度类型</t>
         </is>
       </c>
       <c r="G5" s="44" t="inlineStr">
@@ -5353,27 +5353,27 @@
       </c>
       <c r="I5" s="43" t="inlineStr">
         <is>
-          <t>71/0071 -&gt; 71/0071 -&gt; 70/0070 -&gt; 71/0071；四阶段 integrity=ok、FK=0</t>
+          <t>72/0072 -&gt; 72/0072 -&gt; 71/0071 -&gt; 72/0072；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J5" s="43" t="inlineStr">
         <is>
-          <t>Python 97 passed；Console 26/26；Browser 合同 46/46</t>
+          <t>PRD-079 Python 73；Console 792/792；Browser 合同 9/9；OpenAI 28；FinOps/Webhook 26；兼容回归 29</t>
         </is>
       </c>
       <c r="K5" s="43" t="inlineStr">
         <is>
-          <t>.artifacts/prd078-runtime/prd078-runtime-20260814-08</t>
+          <t>.artifacts/prd079-runtime/run-agent4-b72e1d</t>
         </is>
       </c>
       <c r="L5" s="43" t="inlineStr">
         <is>
-          <t>.artifacts/prd078-browser/prd078-browser-final-20260814-36</t>
+          <t>.artifacts/prd079-browser/main-browser-final-20260814-i</t>
         </is>
       </c>
       <c r="M5" s="43" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-078-mobile-enterprise-approval-entry.md；docs/api/approvals.md；docs/testing/PRD-078-tests.md</t>
+          <t>docs/prd/PRD-079-plan-trial-quota-types.md；docs/api/plan-billing.md；docs/testing/PRD-079-tests.md</t>
         </is>
       </c>
       <c r="N5" s="43" t="b">
@@ -5383,7 +5383,7 @@
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>PRD-079</t>
+          <t>PRD-080</t>
         </is>
       </c>
       <c r="B6" s="45" t="inlineStr">
@@ -5403,12 +5403,12 @@
       </c>
       <c r="E6" s="45" t="inlineStr">
         <is>
-          <t>套餐计费</t>
+          <t>账单争议</t>
         </is>
       </c>
       <c r="F6" s="45" t="inlineStr">
         <is>
-          <t>套餐、试用与额度类型</t>
+          <t>账单争议与调整流程</t>
         </is>
       </c>
       <c r="G6" s="46" t="inlineStr">
@@ -5418,32 +5418,32 @@
       </c>
       <c r="H6" s="45" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="I6" s="45" t="inlineStr">
         <is>
-          <t>72/0072 -&gt; 72/0072 -&gt; 71/0071 -&gt; 72/0072；四阶段 integrity=ok、FK=0</t>
+          <t>73/0073 -&gt; 73/0073 -&gt; 72/0072 -&gt; 73/0073；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J6" s="45" t="inlineStr">
         <is>
-          <t>PRD-079 Python 73；Console 792/792；Browser 合同 9/9；OpenAI 28；FinOps/Webhook 26；兼容回归 29</t>
+          <t>PRD-080 Python 58 passed；Console 815/815；Browser 合同 13/13；PRD-078/079 当前链 30 passed</t>
         </is>
       </c>
       <c r="K6" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd079-runtime/run-agent4-b72e1d</t>
+          <t>.artifacts/prd080-runtime/prd080-runtime-final-20260815-05</t>
         </is>
       </c>
       <c r="L6" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd079-browser/main-browser-final-20260814-i</t>
+          <t>.artifacts/prd080-browser/prd080-browser-final-20260815-05</t>
         </is>
       </c>
       <c r="M6" s="45" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-079-plan-trial-quota-types.md；docs/api/plan-billing.md；docs/testing/PRD-079-tests.md</t>
+          <t>docs/prd/PRD-080-billing-dispute-adjustment-workflow.md；docs/api/billing-disputes.md；docs/testing/PRD-080-tests.md</t>
         </is>
       </c>
       <c r="N6" s="45" t="b">
@@ -5453,7 +5453,7 @@
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>PRD-080</t>
+          <t>PRD-081</t>
         </is>
       </c>
       <c r="B7" s="45" t="inlineStr">
@@ -5473,12 +5473,12 @@
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>账单争议</t>
+          <t>Webhook SIEM</t>
         </is>
       </c>
       <c r="F7" s="45" t="inlineStr">
         <is>
-          <t>账单争议与调整流程</t>
+          <t>SIEM/安全事件格式</t>
         </is>
       </c>
       <c r="G7" s="46" t="inlineStr">
@@ -5488,32 +5488,32 @@
       </c>
       <c r="H7" s="45" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="I7" s="45" t="inlineStr">
         <is>
-          <t>73/0073 -&gt; 73/0073 -&gt; 72/0072 -&gt; 73/0073；四阶段 integrity=ok、FK=0</t>
+          <t>74/0074 -&gt; 74/0074 -&gt; 73/0073 -&gt; 74/0074；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J7" s="45" t="inlineStr">
         <is>
-          <t>PRD-080 Python 58 passed；Console 815/815；Browser 合同 13/13；PRD-078/079 当前链 30 passed</t>
+          <t>Shared/Control 34/34；Gateway 36/36；验收合同 9/9；Console 822/822；Browser 合同 5/5</t>
         </is>
       </c>
       <c r="K7" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd080-runtime/prd080-runtime-final-20260815-05</t>
+          <t>.artifacts/prd081-runtime/final-20260816t</t>
         </is>
       </c>
       <c r="L7" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd080-browser/prd080-browser-final-20260815-05</t>
+          <t>.artifacts/prd081-browser/final-20260816q</t>
         </is>
       </c>
       <c r="M7" s="45" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-080-billing-dispute-adjustment-workflow.md；docs/api/billing-disputes.md；docs/testing/PRD-080-tests.md</t>
+          <t>docs/prd/PRD-081-siem-security-event-format.md；docs/api/webhook-siem.md；docs/testing/PRD-081-tests.md</t>
         </is>
       </c>
       <c r="N7" s="45" t="b">
@@ -5523,7 +5523,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="47" t="inlineStr">
         <is>
-          <t>PRD-080 权威证据摘要</t>
+          <t>PRD-081 权威证据摘要</t>
         </is>
       </c>
       <c r="B8" s="1" t="n"/>
@@ -5548,7 +5548,7 @@
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>74174e1a88553644e08a9584e54e1e866206b943873630c86ecf09fe7619bfd7</t>
+          <t>a67a3d330056a14e92aec86a752964d5228fcc28d72ddbb0e83a81c116cb124d</t>
         </is>
       </c>
       <c r="C9" s="52" t="n"/>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="B10" s="51" t="inlineStr">
         <is>
-          <t>a119250da461f04e966c3867f017084d6048eaf53d56877a0fcfef2a653e5193</t>
+          <t>55f131ad4f79d438fdc81720189e77a99f4da5cbf8480204cea38eb9a7e320dc</t>
         </is>
       </c>
       <c r="C10" s="52" t="n"/>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="B11" s="49" t="inlineStr">
         <is>
-          <t>c0d53161ee0c1463c1cd98cd07d0fa58cd18f8a92b62faf42e71d2935bb12a99</t>
+          <t>ea72a95cfd92e0bbc79720001d771027ea394d476585a13a09ee023e72c93740</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>
@@ -5620,7 +5620,7 @@
       </c>
       <c r="B12" s="51" t="inlineStr">
         <is>
-          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终隐私、错误边界、金额聚合复核无未关闭 P0/P1。</t>
+          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终并发、恢复、权限、隐私与证据复核无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="B13" s="49" t="inlineStr">
         <is>
-          <t>Excel 总表第82行、M2/M3第18行、PAGE-113、Webhook format API、SecurityEventPayload、security.event_pushed、TC-0161/0162 共同确认 PRD-081；本次未实现。</t>
+          <t>Excel 总表第83行、M2/M3第19行、PAGE-114、API-372..377、McpServer/McpTool/McpInvocation、mcp.tool_called、TC-0163/0164 共同确认 PRD-082；本次未实现。</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>

</xml_diff>

<commit_message>
feat: complete PRD-082 MCP tool registration permissions
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -18,7 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_开发状态" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12_开发状态'!$A$4:$N$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12_开发状态'!$A$4:$N$8</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -477,8 +477,8 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MetaHubDevStatus" displayName="MetaHubDevStatus" ref="A4:N6" headerRowCount="1">
-  <autoFilter ref="A4:N6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MetaHubDevStatus" displayName="MetaHubDevStatus" ref="A4:N8" headerRowCount="1">
+  <autoFilter ref="A4:N8"/>
   <tableColumns count="14">
     <tableColumn id="1" name="PRD编号"/>
     <tableColumn id="2" name="里程碑"/>
@@ -5179,7 +5179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5221,7 +5221,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-16。PRD-081 已完成；下一条权威未完成项为 PRD-082，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-16。PRD-082 已完成；下一条权威未完成项为 PRD-083，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -5520,59 +5520,105 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="47" t="inlineStr">
-        <is>
-          <t>PRD-081 权威证据摘要</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
-      <c r="J8" s="1" t="n"/>
-      <c r="K8" s="1" t="n"/>
-      <c r="L8" s="1" t="n"/>
-      <c r="M8" s="1" t="n"/>
-      <c r="N8" s="1" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="48" t="inlineStr">
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="45" t="inlineStr">
+        <is>
+          <t>PRD-082</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="inlineStr">
+        <is>
+          <t>M2-企业增强</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t>扩展层</t>
+        </is>
+      </c>
+      <c r="E8" s="45" t="inlineStr">
+        <is>
+          <t>MCP治理基础</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>MCP工具注册与权限</t>
+        </is>
+      </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H8" s="45" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="I8" s="45" t="inlineStr">
+        <is>
+          <t>75/0075 -&gt; 75/0075 -&gt; 74/0074 -&gt; 75/0075；四阶段 integrity=ok、FK=0</t>
+        </is>
+      </c>
+      <c r="J8" s="45" t="inlineStr">
+        <is>
+          <t>Python 146/146；Scheduler 30/30；Runtime contracts 36/36；Browser harness 8/8；Console 846/846；Browser driver 6/6；lint 261 files；Ruff/compile 通过</t>
+        </is>
+      </c>
+      <c r="K8" s="45" t="inlineStr">
+        <is>
+          <t>.artifacts/prd082-runtime/prd082-final-runtime-7</t>
+        </is>
+      </c>
+      <c r="L8" s="45" t="inlineStr">
+        <is>
+          <t>.artifacts/prd082-browser/prd082-page114-20260816-r8</t>
+        </is>
+      </c>
+      <c r="M8" s="45" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-082-mcp-tool-registration-permissions.md；docs/api/mcp-tools.md；docs/testing/PRD-082-tests.md</t>
+        </is>
+      </c>
+      <c r="N8" s="45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="47" t="inlineStr">
+        <is>
+          <t>PRD-082 权威证据摘要</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="n"/>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
+      <c r="H9" s="1" t="n"/>
+      <c r="I9" s="1" t="n"/>
+      <c r="J9" s="1" t="n"/>
+      <c r="K9" s="1" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="48" t="inlineStr">
         <is>
           <t>Runtime JSON SHA-256</t>
         </is>
       </c>
-      <c r="B9" s="49" t="inlineStr">
-        <is>
-          <t>a67a3d330056a14e92aec86a752964d5228fcc28d72ddbb0e83a81c116cb124d</t>
-        </is>
-      </c>
-      <c r="C9" s="52" t="n"/>
-      <c r="D9" s="52" t="n"/>
-      <c r="E9" s="52" t="n"/>
-      <c r="F9" s="52" t="n"/>
-      <c r="G9" s="52" t="n"/>
-      <c r="H9" s="52" t="n"/>
-      <c r="I9" s="52" t="n"/>
-      <c r="J9" s="52" t="n"/>
-      <c r="K9" s="52" t="n"/>
-      <c r="L9" s="52" t="n"/>
-      <c r="M9" s="52" t="n"/>
-      <c r="N9" s="53" t="n"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="50" t="inlineStr">
-        <is>
-          <t>Browser JSON SHA-256</t>
-        </is>
-      </c>
-      <c r="B10" s="51" t="inlineStr">
-        <is>
-          <t>55f131ad4f79d438fdc81720189e77a99f4da5cbf8480204cea38eb9a7e320dc</t>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>15457991d5e1fb5c1b1acc55530d53acd68e74f9fb53bc5a7c3f3c0633b21c21</t>
         </is>
       </c>
       <c r="C10" s="52" t="n"/>
@@ -5589,14 +5635,14 @@
       <c r="N10" s="53" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="48" t="inlineStr">
-        <is>
-          <t>Browser manifest SHA-256</t>
-        </is>
-      </c>
-      <c r="B11" s="49" t="inlineStr">
-        <is>
-          <t>ea72a95cfd92e0bbc79720001d771027ea394d476585a13a09ee023e72c93740</t>
+      <c r="A11" s="50" t="inlineStr">
+        <is>
+          <t>Browser JSON SHA-256</t>
+        </is>
+      </c>
+      <c r="B11" s="51" t="inlineStr">
+        <is>
+          <t>7c9a965af27968769f8294c14a569bb152e27998d4b083f300f51625511360eb</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>
@@ -5613,14 +5659,14 @@
       <c r="N11" s="53" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="50" t="inlineStr">
-        <is>
-          <t>自审结论</t>
-        </is>
-      </c>
-      <c r="B12" s="51" t="inlineStr">
-        <is>
-          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终并发、恢复、权限、隐私与证据复核无未关闭 P0/P1。</t>
+      <c r="A12" s="48" t="inlineStr">
+        <is>
+          <t>Browser manifest SHA-256</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>e387ef1cf76b53b2a886751899ab919b9ea5fd90ca44beb9ec74e953f4eb411c</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>
@@ -5636,15 +5682,15 @@
       <c r="M12" s="52" t="n"/>
       <c r="N12" s="53" t="n"/>
     </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="48" t="inlineStr">
-        <is>
-          <t>下一项依据</t>
-        </is>
-      </c>
-      <c r="B13" s="49" t="inlineStr">
-        <is>
-          <t>Excel 总表第83行、M2/M3第19行、PAGE-114、API-372..377、McpServer/McpTool/McpInvocation、mcp.tool_called、TC-0163/0164 共同确认 PRD-082；本次未实现。</t>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>自审结论</t>
+        </is>
+      </c>
+      <c r="B13" s="51" t="inlineStr">
+        <is>
+          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终并发、恢复、权限、隐私与证据复核无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>
@@ -5660,15 +5706,15 @@
       <c r="M13" s="52" t="n"/>
       <c r="N13" s="53" t="n"/>
     </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="50" t="inlineStr">
-        <is>
-          <t>总体状态</t>
-        </is>
-      </c>
-      <c r="B14" s="51" t="inlineStr">
-        <is>
-          <t>all_108_prds_complete=false</t>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="48" t="inlineStr">
+        <is>
+          <t>下一项依据</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Excel 总表第84行、M2/M3第20行、PAGE-115、API-378..382、McpNetworkPolicy/OBJ-114、mcp.network_blocked、TC-0165/0166 共同确认 PRD-083；本次未实现。</t>
         </is>
       </c>
       <c r="C14" s="52" t="n"/>
@@ -5684,15 +5730,39 @@
       <c r="M14" s="52" t="n"/>
       <c r="N14" s="53" t="n"/>
     </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>总体状态</t>
+        </is>
+      </c>
+      <c r="B15" s="51" t="inlineStr">
+        <is>
+          <t>all_108_prds_complete=false</t>
+        </is>
+      </c>
+      <c r="C15" s="52" t="n"/>
+      <c r="D15" s="52" t="n"/>
+      <c r="E15" s="52" t="n"/>
+      <c r="F15" s="52" t="n"/>
+      <c r="G15" s="52" t="n"/>
+      <c r="H15" s="52" t="n"/>
+      <c r="I15" s="52" t="n"/>
+      <c r="J15" s="52" t="n"/>
+      <c r="K15" s="52" t="n"/>
+      <c r="L15" s="52" t="n"/>
+      <c r="M15" s="52" t="n"/>
+      <c r="N15" s="53" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N6"/>
+  <autoFilter ref="A4:N8"/>
   <mergeCells count="9">
+    <mergeCell ref="A9:N9"/>
     <mergeCell ref="B14:N14"/>
-    <mergeCell ref="A8:N8"/>
-    <mergeCell ref="B9:N9"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="B12:N12"/>
     <mergeCell ref="B13:N13"/>
+    <mergeCell ref="B15:N15"/>
     <mergeCell ref="B11:N11"/>
     <mergeCell ref="B10:N10"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
feat: complete PRD-083 third-party MCP sandbox network ACL
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -477,7 +477,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MetaHubDevStatus" displayName="MetaHubDevStatus" ref="A4:N8" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MetaHubDevStatus" displayName="MetaHubDevStatus" ref="A4:N9" headerRowCount="1">
   <autoFilter ref="A4:N8"/>
   <tableColumns count="14">
     <tableColumn id="1" name="PRD编号"/>
@@ -5179,7 +5179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5221,7 +5221,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-16。PRD-082 已完成；下一条权威未完成项为 PRD-083，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-16。PRD-083 已完成；下一条权威未完成项为 PRD-084，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -5238,6 +5238,7 @@
       <c r="M2" s="1" t="n"/>
       <c r="N2" s="1" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -5590,59 +5591,105 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="47" t="inlineStr">
-        <is>
-          <t>PRD-082 权威证据摘要</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="1" t="n"/>
-      <c r="J9" s="1" t="n"/>
-      <c r="K9" s="1" t="n"/>
-      <c r="L9" s="1" t="n"/>
-      <c r="M9" s="1" t="n"/>
-      <c r="N9" s="1" t="n"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="48" t="inlineStr">
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>PRD-083</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>M2-企业增强</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>扩展层</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="inlineStr">
+        <is>
+          <t>MCP沙箱</t>
+        </is>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>第三方MCP沙箱网络ACL</t>
+        </is>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H9" s="45" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="I9" s="45" t="inlineStr">
+        <is>
+          <t>76/0076 -&gt; 76/0076 -&gt; 75/0075 -&gt; 76/0076；四阶段 integrity=ok、FK=0</t>
+        </is>
+      </c>
+      <c r="J9" s="45" t="inlineStr">
+        <is>
+          <t>Shared 9/9；Worker 28/28；Scheduler 20/20；0076/Compose 17/17；相邻 MCP 35/35；Console 33/33；验收合同 62/62；Browser driver 6/6；Ruff/lint 通过</t>
+        </is>
+      </c>
+      <c r="K9" s="45" t="inlineStr">
+        <is>
+          <t>.artifacts/prd083-runtime/prd083-final-20260816-ac</t>
+        </is>
+      </c>
+      <c r="L9" s="45" t="inlineStr">
+        <is>
+          <t>.artifacts/prd083-browser/prd083-final-20260816-f</t>
+        </is>
+      </c>
+      <c r="M9" s="45" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-083-third-party-mcp-sandbox-network-acl.md；docs/api/mcp-tools.md；docs/deployment/single-node-compose.md；docs/testing/PRD-083-tests.md</t>
+        </is>
+      </c>
+      <c r="N9" s="45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="47" t="inlineStr">
+        <is>
+          <t>PRD-083 权威证据摘要</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" s="1" t="n"/>
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Runtime JSON SHA-256</t>
         </is>
       </c>
-      <c r="B10" s="49" t="inlineStr">
-        <is>
-          <t>15457991d5e1fb5c1b1acc55530d53acd68e74f9fb53bc5a7c3f3c0633b21c21</t>
-        </is>
-      </c>
-      <c r="C10" s="52" t="n"/>
-      <c r="D10" s="52" t="n"/>
-      <c r="E10" s="52" t="n"/>
-      <c r="F10" s="52" t="n"/>
-      <c r="G10" s="52" t="n"/>
-      <c r="H10" s="52" t="n"/>
-      <c r="I10" s="52" t="n"/>
-      <c r="J10" s="52" t="n"/>
-      <c r="K10" s="52" t="n"/>
-      <c r="L10" s="52" t="n"/>
-      <c r="M10" s="52" t="n"/>
-      <c r="N10" s="53" t="n"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="50" t="inlineStr">
-        <is>
-          <t>Browser JSON SHA-256</t>
-        </is>
-      </c>
-      <c r="B11" s="51" t="inlineStr">
-        <is>
-          <t>7c9a965af27968769f8294c14a569bb152e27998d4b083f300f51625511360eb</t>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>c5ffb99b15ff2156d26408b08c4f8acd2c4ec07610a06799dddfe471b23d0047</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>
@@ -5659,14 +5706,14 @@
       <c r="N11" s="53" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="48" t="inlineStr">
-        <is>
-          <t>Browser manifest SHA-256</t>
-        </is>
-      </c>
-      <c r="B12" s="49" t="inlineStr">
-        <is>
-          <t>e387ef1cf76b53b2a886751899ab919b9ea5fd90ca44beb9ec74e953f4eb411c</t>
+      <c r="A12" s="50" t="inlineStr">
+        <is>
+          <t>Browser JSON SHA-256</t>
+        </is>
+      </c>
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t>30685f52892ae64838cca4c32c1caa044b974d311d8e0425016bffdc8c61ae94</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>
@@ -5683,14 +5730,14 @@
       <c r="N12" s="53" t="n"/>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="50" t="inlineStr">
-        <is>
-          <t>自审结论</t>
-        </is>
-      </c>
-      <c r="B13" s="51" t="inlineStr">
-        <is>
-          <t>两轮编码前自审和两轮实现后自审均已完成并修正；最终并发、恢复、权限、隐私与证据复核无未关闭 P0/P1。</t>
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>Browser manifest SHA-256</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>0c59fee846b45b54461dc00d7c86c2591f47ebf9b87248cb3850128d80830044</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>
@@ -5706,15 +5753,15 @@
       <c r="M13" s="52" t="n"/>
       <c r="N13" s="53" t="n"/>
     </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="48" t="inlineStr">
-        <is>
-          <t>下一项依据</t>
-        </is>
-      </c>
-      <c r="B14" s="49" t="inlineStr">
-        <is>
-          <t>Excel 总表第84行、M2/M3第20行、PAGE-115、API-378..382、McpNetworkPolicy/OBJ-114、mcp.network_blocked、TC-0165/0166 共同确认 PRD-083；本次未实现。</t>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="50" t="inlineStr">
+        <is>
+          <t>自审结论</t>
+        </is>
+      </c>
+      <c r="B14" s="51" t="inlineStr">
+        <is>
+          <t>两轮编码前自审和两轮实现后深审均已完成并修正；最终权限、租户、网络、恢复、并发、隐私与证据复核无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C14" s="52" t="n"/>
@@ -5730,15 +5777,15 @@
       <c r="M14" s="52" t="n"/>
       <c r="N14" s="53" t="n"/>
     </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="50" t="inlineStr">
-        <is>
-          <t>总体状态</t>
-        </is>
-      </c>
-      <c r="B15" s="51" t="inlineStr">
-        <is>
-          <t>all_108_prds_complete=false</t>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>下一项依据</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Excel 总表第85行、M2/M3第21行、PAGE-116、API-383..388、OBJ-115、EVT-096、TC-0167/0168 共同确认 PRD-084；本次未实现。</t>
         </is>
       </c>
       <c r="C15" s="52" t="n"/>
@@ -5754,17 +5801,41 @@
       <c r="M15" s="52" t="n"/>
       <c r="N15" s="53" t="n"/>
     </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="50" t="inlineStr">
+        <is>
+          <t>总体状态</t>
+        </is>
+      </c>
+      <c r="B16" s="51" t="inlineStr">
+        <is>
+          <t>all_108_prds_complete=false</t>
+        </is>
+      </c>
+      <c r="C16" s="52" t="n"/>
+      <c r="D16" s="52" t="n"/>
+      <c r="E16" s="52" t="n"/>
+      <c r="F16" s="52" t="n"/>
+      <c r="G16" s="52" t="n"/>
+      <c r="H16" s="52" t="n"/>
+      <c r="I16" s="52" t="n"/>
+      <c r="J16" s="52" t="n"/>
+      <c r="K16" s="52" t="n"/>
+      <c r="L16" s="52" t="n"/>
+      <c r="M16" s="52" t="n"/>
+      <c r="N16" s="53" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A4:N8"/>
   <mergeCells count="9">
-    <mergeCell ref="A9:N9"/>
     <mergeCell ref="B14:N14"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="B12:N12"/>
     <mergeCell ref="B13:N13"/>
     <mergeCell ref="B15:N15"/>
+    <mergeCell ref="A10:N10"/>
     <mergeCell ref="B11:N11"/>
-    <mergeCell ref="B10:N10"/>
+    <mergeCell ref="B16:N16"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: complete PRD-084 local model endpoint access
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5221,7 +5221,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-16。PRD-083 已完成；下一条权威未完成项为 PRD-084，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-17。PRD-084 已完成；下一条权威未完成项为 PRD-085，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -5238,7 +5238,6 @@
       <c r="M2" s="1" t="n"/>
       <c r="N2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -5314,7 +5313,7 @@
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="43" t="inlineStr">
         <is>
-          <t>PRD-079</t>
+          <t>PRD-080</t>
         </is>
       </c>
       <c r="B5" s="43" t="inlineStr">
@@ -5334,12 +5333,12 @@
       </c>
       <c r="E5" s="43" t="inlineStr">
         <is>
-          <t>套餐计费</t>
+          <t>账单争议</t>
         </is>
       </c>
       <c r="F5" s="43" t="inlineStr">
         <is>
-          <t>套餐、试用与额度类型</t>
+          <t>账单争议与调整流程</t>
         </is>
       </c>
       <c r="G5" s="44" t="inlineStr">
@@ -5349,32 +5348,32 @@
       </c>
       <c r="H5" s="43" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="I5" s="43" t="inlineStr">
         <is>
-          <t>72/0072 -&gt; 72/0072 -&gt; 71/0071 -&gt; 72/0072；四阶段 integrity=ok、FK=0</t>
+          <t>73/0073 -&gt; 73/0073 -&gt; 72/0072 -&gt; 73/0073；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J5" s="43" t="inlineStr">
         <is>
-          <t>PRD-079 Python 73；Console 792/792；Browser 合同 9/9；OpenAI 28；FinOps/Webhook 26；兼容回归 29</t>
+          <t>PRD-080 Python 58 passed；Console 815/815；Browser 合同 13/13；PRD-078/079 当前链 30 passed</t>
         </is>
       </c>
       <c r="K5" s="43" t="inlineStr">
         <is>
-          <t>.artifacts/prd079-runtime/run-agent4-b72e1d</t>
+          <t>.artifacts/prd080-runtime/prd080-runtime-final-20260815-05</t>
         </is>
       </c>
       <c r="L5" s="43" t="inlineStr">
         <is>
-          <t>.artifacts/prd079-browser/main-browser-final-20260814-i</t>
+          <t>.artifacts/prd080-browser/prd080-browser-final-20260815-05</t>
         </is>
       </c>
       <c r="M5" s="43" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-079-plan-trial-quota-types.md；docs/api/plan-billing.md；docs/testing/PRD-079-tests.md</t>
+          <t>docs/prd/PRD-080-billing-dispute-adjustment-workflow.md；docs/api/billing-disputes.md；docs/testing/PRD-080-tests.md</t>
         </is>
       </c>
       <c r="N5" s="43" t="b">
@@ -5384,7 +5383,7 @@
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>PRD-080</t>
+          <t>PRD-081</t>
         </is>
       </c>
       <c r="B6" s="45" t="inlineStr">
@@ -5404,12 +5403,12 @@
       </c>
       <c r="E6" s="45" t="inlineStr">
         <is>
-          <t>账单争议</t>
+          <t>Webhook SIEM</t>
         </is>
       </c>
       <c r="F6" s="45" t="inlineStr">
         <is>
-          <t>账单争议与调整流程</t>
+          <t>SIEM/安全事件格式</t>
         </is>
       </c>
       <c r="G6" s="46" t="inlineStr">
@@ -5419,32 +5418,32 @@
       </c>
       <c r="H6" s="45" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="I6" s="45" t="inlineStr">
         <is>
-          <t>73/0073 -&gt; 73/0073 -&gt; 72/0072 -&gt; 73/0073；四阶段 integrity=ok、FK=0</t>
+          <t>74/0074 -&gt; 74/0074 -&gt; 73/0073 -&gt; 74/0074；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J6" s="45" t="inlineStr">
         <is>
-          <t>PRD-080 Python 58 passed；Console 815/815；Browser 合同 13/13；PRD-078/079 当前链 30 passed</t>
+          <t>Shared/Control 34/34；Gateway 36/36；验收合同 9/9；Console 822/822；Browser 合同 5/5</t>
         </is>
       </c>
       <c r="K6" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd080-runtime/prd080-runtime-final-20260815-05</t>
+          <t>.artifacts/prd081-runtime/final-20260816t</t>
         </is>
       </c>
       <c r="L6" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd080-browser/prd080-browser-final-20260815-05</t>
+          <t>.artifacts/prd081-browser/final-20260816q</t>
         </is>
       </c>
       <c r="M6" s="45" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-080-billing-dispute-adjustment-workflow.md；docs/api/billing-disputes.md；docs/testing/PRD-080-tests.md</t>
+          <t>docs/prd/PRD-081-siem-security-event-format.md；docs/api/webhook-siem.md；docs/testing/PRD-081-tests.md</t>
         </is>
       </c>
       <c r="N6" s="45" t="b">
@@ -5454,7 +5453,7 @@
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>PRD-081</t>
+          <t>PRD-082</t>
         </is>
       </c>
       <c r="B7" s="45" t="inlineStr">
@@ -5474,12 +5473,12 @@
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>Webhook SIEM</t>
+          <t>MCP治理基础</t>
         </is>
       </c>
       <c r="F7" s="45" t="inlineStr">
         <is>
-          <t>SIEM/安全事件格式</t>
+          <t>MCP工具注册与权限</t>
         </is>
       </c>
       <c r="G7" s="46" t="inlineStr">
@@ -5494,27 +5493,27 @@
       </c>
       <c r="I7" s="45" t="inlineStr">
         <is>
-          <t>74/0074 -&gt; 74/0074 -&gt; 73/0073 -&gt; 74/0074；四阶段 integrity=ok、FK=0</t>
+          <t>75/0075 -&gt; 75/0075 -&gt; 74/0074 -&gt; 75/0075；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J7" s="45" t="inlineStr">
         <is>
-          <t>Shared/Control 34/34；Gateway 36/36；验收合同 9/9；Console 822/822；Browser 合同 5/5</t>
+          <t>Python 146/146；Scheduler 30/30；Runtime contracts 36/36；Browser harness 8/8；Console 846/846；Browser driver 6/6；lint 261 files；Ruff/compile 通过</t>
         </is>
       </c>
       <c r="K7" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd081-runtime/final-20260816t</t>
+          <t>.artifacts/prd082-runtime/prd082-final-runtime-7</t>
         </is>
       </c>
       <c r="L7" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd081-browser/final-20260816q</t>
+          <t>.artifacts/prd082-browser/prd082-page114-20260816-r8</t>
         </is>
       </c>
       <c r="M7" s="45" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-081-siem-security-event-format.md；docs/api/webhook-siem.md；docs/testing/PRD-081-tests.md</t>
+          <t>docs/prd/PRD-082-mcp-tool-registration-permissions.md；docs/api/mcp-tools.md；docs/testing/PRD-082-tests.md</t>
         </is>
       </c>
       <c r="N7" s="45" t="b">
@@ -5524,7 +5523,7 @@
     <row r="8" ht="54" customHeight="1">
       <c r="A8" s="45" t="inlineStr">
         <is>
-          <t>PRD-082</t>
+          <t>PRD-083</t>
         </is>
       </c>
       <c r="B8" s="45" t="inlineStr">
@@ -5544,12 +5543,12 @@
       </c>
       <c r="E8" s="45" t="inlineStr">
         <is>
-          <t>MCP治理基础</t>
+          <t>MCP沙箱</t>
         </is>
       </c>
       <c r="F8" s="45" t="inlineStr">
         <is>
-          <t>MCP工具注册与权限</t>
+          <t>第三方MCP沙箱网络ACL</t>
         </is>
       </c>
       <c r="G8" s="46" t="inlineStr">
@@ -5564,27 +5563,27 @@
       </c>
       <c r="I8" s="45" t="inlineStr">
         <is>
-          <t>75/0075 -&gt; 75/0075 -&gt; 74/0074 -&gt; 75/0075；四阶段 integrity=ok、FK=0</t>
+          <t>76/0076 -&gt; 76/0076 -&gt; 75/0075 -&gt; 76/0076；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J8" s="45" t="inlineStr">
         <is>
-          <t>Python 146/146；Scheduler 30/30；Runtime contracts 36/36；Browser harness 8/8；Console 846/846；Browser driver 6/6；lint 261 files；Ruff/compile 通过</t>
+          <t>Shared 9/9；Worker 28/28；Scheduler 20/20；0076/Compose 17/17；相邻 MCP 35/35；Console 33/33；验收合同 62/62；Browser driver 6/6；Ruff/lint 通过</t>
         </is>
       </c>
       <c r="K8" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd082-runtime/prd082-final-runtime-7</t>
+          <t>.artifacts/prd083-runtime/prd083-final-20260816-ac</t>
         </is>
       </c>
       <c r="L8" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd082-browser/prd082-page114-20260816-r8</t>
+          <t>.artifacts/prd083-browser/prd083-final-20260816-f</t>
         </is>
       </c>
       <c r="M8" s="45" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-082-mcp-tool-registration-permissions.md；docs/api/mcp-tools.md；docs/testing/PRD-082-tests.md</t>
+          <t>docs/prd/PRD-083-third-party-mcp-sandbox-network-acl.md；docs/api/mcp-tools.md；docs/deployment/single-node-compose.md；docs/testing/PRD-083-tests.md</t>
         </is>
       </c>
       <c r="N8" s="45" t="b">
@@ -5594,7 +5593,7 @@
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="45" t="inlineStr">
         <is>
-          <t>PRD-083</t>
+          <t>PRD-084</t>
         </is>
       </c>
       <c r="B9" s="45" t="inlineStr">
@@ -5614,12 +5613,12 @@
       </c>
       <c r="E9" s="45" t="inlineStr">
         <is>
-          <t>MCP沙箱</t>
+          <t>本地模型</t>
         </is>
       </c>
       <c r="F9" s="45" t="inlineStr">
         <is>
-          <t>第三方MCP沙箱网络ACL</t>
+          <t>本地模型Endpoint接入</t>
         </is>
       </c>
       <c r="G9" s="46" t="inlineStr">
@@ -5629,32 +5628,32 @@
       </c>
       <c r="H9" s="45" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="I9" s="45" t="inlineStr">
         <is>
-          <t>76/0076 -&gt; 76/0076 -&gt; 75/0075 -&gt; 76/0076；四阶段 integrity=ok、FK=0</t>
+          <t>77/0077 -&gt; 77/0077 -&gt; 76/0076 -&gt; 77/0077；四阶段 integrity=ok、FK=0</t>
         </is>
       </c>
       <c r="J9" s="45" t="inlineStr">
         <is>
-          <t>Shared 9/9；Worker 28/28；Scheduler 20/20；0076/Compose 17/17；相邻 MCP 35/35；Console 33/33；验收合同 62/62；Browser driver 6/6；Ruff/lint 通过</t>
+          <t>联合专项 56/56；持久层/网络/取消 20/20；Shared 116/116；Gateway 74/74；Adapter v2 103/103；Control 12/12；Console 876/876；Runtime 8/8；Browser harness 7/7；driver 6/6；Ruff/lint 通过</t>
         </is>
       </c>
       <c r="K9" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd083-runtime/prd083-final-20260816-ac</t>
+          <t>.artifacts/prd084-runtime/20260816T183036Z-c60eb988.json</t>
         </is>
       </c>
       <c r="L9" s="45" t="inlineStr">
         <is>
-          <t>.artifacts/prd083-browser/prd083-final-20260816-f</t>
+          <t>.artifacts/prd084-browser/final-20260817-01</t>
         </is>
       </c>
       <c r="M9" s="45" t="inlineStr">
         <is>
-          <t>docs/prd/PRD-083-third-party-mcp-sandbox-network-acl.md；docs/api/mcp-tools.md；docs/deployment/single-node-compose.md；docs/testing/PRD-083-tests.md</t>
+          <t>docs/prd/PRD-084-local-model-endpoint-access.md；docs/api/local-model-endpoints.md；docs/deployment/single-node-compose.md；docs/testing/PRD-084-tests.md</t>
         </is>
       </c>
       <c r="N9" s="45" t="b">
@@ -5664,7 +5663,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="47" t="inlineStr">
         <is>
-          <t>PRD-083 权威证据摘要</t>
+          <t>PRD-084 权威证据摘要</t>
         </is>
       </c>
       <c r="B10" s="1" t="n"/>
@@ -5689,7 +5688,7 @@
       </c>
       <c r="B11" s="49" t="inlineStr">
         <is>
-          <t>c5ffb99b15ff2156d26408b08c4f8acd2c4ec07610a06799dddfe471b23d0047</t>
+          <t>f226d7665714c6af335c72ae64e33392976337ce7a1e8850319384c8ffdbfddc</t>
         </is>
       </c>
       <c r="C11" s="52" t="n"/>
@@ -5713,7 +5712,7 @@
       </c>
       <c r="B12" s="51" t="inlineStr">
         <is>
-          <t>30685f52892ae64838cca4c32c1caa044b974d311d8e0425016bffdc8c61ae94</t>
+          <t>f1c6eaf61b496956326cd56974058a9250faf8af20c23816f1f9eff9a949507e</t>
         </is>
       </c>
       <c r="C12" s="52" t="n"/>
@@ -5737,7 +5736,7 @@
       </c>
       <c r="B13" s="49" t="inlineStr">
         <is>
-          <t>0c59fee846b45b54461dc00d7c86c2591f47ebf9b87248cb3850128d80830044</t>
+          <t>9a20078068521d2c3e1ac33c838e7edbba5060f112617c5babba28fc66290f13</t>
         </is>
       </c>
       <c r="C13" s="52" t="n"/>
@@ -5761,7 +5760,7 @@
       </c>
       <c r="B14" s="51" t="inlineStr">
         <is>
-          <t>两轮编码前自审和两轮实现后深审均已完成并修正；最终权限、租户、网络、恢复、并发、隐私与证据复核无未关闭 P0/P1。</t>
+          <t>两轮编码前自审和两轮实现后深审均已完成并修正；最终 tenant/RBAC、网络、恢复、取消、用量、事件、隐私与证据复核无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C14" s="52" t="n"/>
@@ -5785,7 +5784,7 @@
       </c>
       <c r="B15" s="49" t="inlineStr">
         <is>
-          <t>Excel 总表第85行、M2/M3第21行、PAGE-116、API-383..388、OBJ-115、EVT-096、TC-0167/0168 共同确认 PRD-084；本次未实现。</t>
+          <t>Excel 总表第86行、M2/M3第22行、PAGE-117、API-389..391、OBJ-116、EVT-097、TC-0169/0170 共同确认 PRD-085；本次未实现。</t>
         </is>
       </c>
       <c r="C15" s="52" t="n"/>

</xml_diff>

<commit_message>
feat: complete PRD-086 customer health score
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5173,7 +5173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="2"/>
@@ -5201,7 +5201,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-17。PRD-085 已完成；下一条权威未完成项为 PRD-086，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-17。PRD-086 已完成；下一条权威未完成项为 PRD-087，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
     </row>
@@ -5697,46 +5697,92 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>PRD-085 权威证据摘要</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Runtime JSON SHA-256</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>9bc26bcd9dc04a18b9628be5a689fe9492ee2e4ed99f6a623dffe36397ee61d6</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="21" t="n"/>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="21" t="n"/>
-      <c r="L12" s="21" t="n"/>
-      <c r="M12" s="21" t="n"/>
-      <c r="N12" s="22" t="n"/>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>PRD-086</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>M2-企业增强</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>扩展层</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>客户健康</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>客户健康评分</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>79/0079 -&gt; 79/0079 -&gt; 78/0078 -&gt; 79/0079；四阶段 integrity=ok、FK=0</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Shared 36/36；Control 7/7；Migration 12/12；Console PAGE-118 14/14；Python 相邻 92/92；Console 受影响 61/61；lint 279 files；真实 API 200/401/403/422/503、纯读计数 3/3/3 不变；1280/1440/390 四状态 Browser 通过；Ruff/compile/diff 通过</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>.artifacts/prd086-runtime/prd086-live-20260817-05</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>.artifacts/prd086-runtime/prd086-live-20260817-06</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-086-customer-health-score.md；docs/api/customer-health.md；docs/testing/PRD-086-tests.md</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>PRD-086 权威证据摘要</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Browser JSON SHA-256</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>2ba160c3b7351ff1b9771ac1d2bd1bba9bcfb06b90e94caa3463484b92a881f9</t>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Runtime/API JSON SHA-256</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>runtime=56fd2262be07a3b8f76a3cdc71675091f033f10576ad38c13fa96e8393ff9756；api=80bb42199b38d095ea65b8117a10bc091c9315e263046d53d623cd43ef662df9</t>
         </is>
       </c>
       <c r="C13" s="21" t="n"/>
@@ -5755,12 +5801,12 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Browser manifest SHA-256</t>
+          <t>Browser JSON SHA-256</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>bc51513b7ed3b20af628121c1d49adcc7a5fedb6d4a04156875d113591be49a1</t>
+          <t>215c73b2ab40064f06094d8bfdda86a8878e6a6a050d08c92d0dd475f8bac74f</t>
         </is>
       </c>
       <c r="C14" s="21" t="n"/>
@@ -5777,14 +5823,14 @@
       <c r="N14" s="22" t="n"/>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>自审结论</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>编码前两轮与实现后两轮自审闭环；tenant/RBAC、来源/恢复、整数口径、日志/隐私、定向中文注释和 Chromium owner 清理均通过，无未关闭 P0/P1。</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>四张 PNG SHA-256</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>healthy=6ded26bde4a6035e27c08c78cf898e461ce53db5436588dd92df6643a958fafc；risk=6df5e8d9f342a77aeadb44f8d0e010903a76d7640244e5dd2d5c922cf3d5f422；no_samples=373824dec96d875d71c3c77f5033650fc81a0401f10867c5e11a75edf875074d；isolation=640ef0d2fec161da736de1dc637965d35303673188baffc01cf63f2e90e90c27</t>
         </is>
       </c>
       <c r="C15" s="21" t="n"/>
@@ -5800,15 +5846,15 @@
       <c r="M15" s="21" t="n"/>
       <c r="N15" s="22" t="n"/>
     </row>
-    <row r="16" ht="46" customHeight="1">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>下一项依据</t>
+          <t>自审结论</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Excel 总表第87行、M2/M3第23行、PAGE-118、API-392/393、OBJ-117、EVT-098、TC-0171/0172 共同确认 PRD-086；本次未实现。</t>
+          <t>编码前两轮自审闭环；tenant/RBAC、纯读 GET、整数公式、Scheduler/outbox、日志/隐私和双视口均通过，无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C16" s="21" t="n"/>
@@ -5824,15 +5870,15 @@
       <c r="M16" s="21" t="n"/>
       <c r="N16" s="22" t="n"/>
     </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>总体状态</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>all_108_prds_complete=false</t>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>下一项依据</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Excel 总表第88行、M2/M3第24行、PAGE-119、API-394..399、OBJ-118..120、EVT-099、TC-0173/0174 共同确认 PRD-087；本次未实现。</t>
         </is>
       </c>
       <c r="C17" s="21" t="n"/>
@@ -5848,15 +5894,39 @@
       <c r="M17" s="21" t="n"/>
       <c r="N17" s="22" t="n"/>
     </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>总体状态</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>all_108_prds_complete=false</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="21" t="n"/>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="21" t="n"/>
+      <c r="J18" s="21" t="n"/>
+      <c r="K18" s="21" t="n"/>
+      <c r="L18" s="21" t="n"/>
+      <c r="M18" s="21" t="n"/>
+      <c r="N18" s="22" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A4:N10"/>
   <mergeCells count="9">
     <mergeCell ref="B14:N14"/>
+    <mergeCell ref="A12:N12"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="B17:N17"/>
-    <mergeCell ref="B12:N12"/>
+    <mergeCell ref="B18:N18"/>
     <mergeCell ref="B13:N13"/>
-    <mergeCell ref="A11:N11"/>
     <mergeCell ref="B15:N15"/>
     <mergeCell ref="B16:N16"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
feat: complete PRD-087 channel partner white-label portal
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -21,7 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_开发状态" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12_开发状态'!$A$4:$N$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12_开发状态'!$A$4:$N$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -5173,7 +5173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="2"/>
@@ -5201,7 +5201,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-17。PRD-086 已完成；下一条权威未完成项为 PRD-087，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
+          <t>更新时间：2026-08-17。PRD-087 已完成；下一条权威未完成项为 PRD-088，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
         </is>
       </c>
     </row>
@@ -5767,36 +5767,82 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>PRD-086 权威证据摘要</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Runtime/API JSON SHA-256</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>runtime=56fd2262be07a3b8f76a3cdc71675091f033f10576ad38c13fa96e8393ff9756；api=80bb42199b38d095ea65b8117a10bc091c9315e263046d53d623cd43ef662df9</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="21" t="n"/>
-      <c r="H13" s="21" t="n"/>
-      <c r="I13" s="21" t="n"/>
-      <c r="J13" s="21" t="n"/>
-      <c r="K13" s="21" t="n"/>
-      <c r="L13" s="21" t="n"/>
-      <c r="M13" s="21" t="n"/>
-      <c r="N13" s="22" t="n"/>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>PRD-087</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>M2-企业增强</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>扩展层</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>伙伴门户</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>渠道伙伴与白标门户</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>80/0080 -&gt; 80/0080 -&gt; 79/0079 -&gt; 80/0080；四阶段 integrity=ok、FK=0</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Python 联合 53/53；Shared 相邻 81/81；Control 相邻 17/17；PAGE-119 Console 18/18；Console 全量 926/926；lint 286 files；真实 Browser 19/19 请求响应、双租户、动态撤权、未授权零预取、四张 PNG、Ruff/compile/diff 通过</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>.artifacts/prd087-browser/page119-final-20260817-r17/browser-acceptance.json</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>.artifacts/prd087-browser/page119-final-20260817-r17</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-087-channel-partner-white-label-portal.md；docs/api/partner-portal.md；docs/testing/PRD-087-tests.md</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>PRD-087 权威证据摘要</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
@@ -5806,7 +5852,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>215c73b2ab40064f06094d8bfdda86a8878e6a6a050d08c92d0dd475f8bac74f</t>
+          <t>b74797106b0f8859b9a676236c357ba10280d2d0fa8f82a88ed66abe48fb17dc</t>
         </is>
       </c>
       <c r="C14" s="21" t="n"/>
@@ -5825,12 +5871,12 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>四张 PNG SHA-256</t>
+          <t>Browser manifest SHA-256</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>healthy=6ded26bde4a6035e27c08c78cf898e461ce53db5436588dd92df6643a958fafc；risk=6df5e8d9f342a77aeadb44f8d0e010903a76d7640244e5dd2d5c922cf3d5f422；no_samples=373824dec96d875d71c3c77f5033650fc81a0401f10867c5e11a75edf875074d；isolation=640ef0d2fec161da736de1dc637965d35303673188baffc01cf63f2e90e90c27</t>
+          <t>d7c91394e60d828f8990b2531cca9c34bb76180b2f9c89271ecb3098f90a6688</t>
         </is>
       </c>
       <c r="C15" s="21" t="n"/>
@@ -5849,12 +5895,12 @@
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>自审结论</t>
+          <t>四张 PNG SHA-256</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>编码前两轮自审闭环；tenant/RBAC、纯读 GET、整数公式、Scheduler/outbox、日志/隐私和双视口均通过，无未关闭 P0/P1。</t>
+          <t>setup=cb3b4d6c4e1efe5085116d64d7dadab65bdda1c485d0f0f7236585a4ffc13902；ready=1b607b22d1a614abecfb514bb7b304429ae5a8c328546e836fa65af5ae4fe82c；commission=f96fc8bb1a5d096d15c4147296e63e9269273083bfcf6d67e3d6c0bbd478d5bb；isolation=883548bf8be8fdc64794f49f6af821d22e0f7ad52547f5844981d86fc59c3e64</t>
         </is>
       </c>
       <c r="C16" s="21" t="n"/>
@@ -5870,15 +5916,15 @@
       <c r="M16" s="21" t="n"/>
       <c r="N16" s="22" t="n"/>
     </row>
-    <row r="17" ht="46" customHeight="1">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>下一项依据</t>
+          <t>自审结论</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Excel 总表第88行、M2/M3第24行、PAGE-119、API-394..399、OBJ-118..120、EVT-099、TC-0173/0174 共同确认 PRD-087；本次未实现。</t>
+          <t>编码前两轮自审闭环；tenant/RBAC、幂等/CAS、分润并发/cutoff、EVT-099 恢复、附件隐私、动态撤权和双租户均通过，无未关闭 P0/P1。</t>
         </is>
       </c>
       <c r="C17" s="21" t="n"/>
@@ -5894,15 +5940,15 @@
       <c r="M17" s="21" t="n"/>
       <c r="N17" s="22" t="n"/>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="46" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>总体状态</t>
+          <t>下一项依据</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>all_108_prds_complete=false</t>
+          <t>Excel 总表第89行、M2/M3第25行、PAGE-120、API-400/401、OBJ-121、EVT-100、TC-0175/0176 共同确认 PRD-088；本次未实现。</t>
         </is>
       </c>
       <c r="C18" s="21" t="n"/>
@@ -5918,15 +5964,39 @@
       <c r="M18" s="21" t="n"/>
       <c r="N18" s="22" t="n"/>
     </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>总体状态</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>all_108_prds_complete=false</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="21" t="n"/>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21" t="n"/>
+      <c r="M19" s="21" t="n"/>
+      <c r="N19" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N10"/>
+  <autoFilter ref="A4:N12"/>
   <mergeCells count="9">
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="B14:N14"/>
-    <mergeCell ref="A12:N12"/>
     <mergeCell ref="A2:N2"/>
+    <mergeCell ref="B18:N18"/>
     <mergeCell ref="B17:N17"/>
-    <mergeCell ref="B18:N18"/>
-    <mergeCell ref="B13:N13"/>
+    <mergeCell ref="B19:N19"/>
     <mergeCell ref="B15:N15"/>
     <mergeCell ref="B16:N16"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
feat: complete PRD-088 tenant white-label branding
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5173,7 +5173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="2"/>
@@ -5201,10 +5201,11 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-17。PRD-087 已完成；下一条权威未完成项为 PRD-088，但本次未启动。总体状态保持 all_108_prds_complete=false。</t>
-        </is>
-      </c>
-    </row>
+          <t>更新时间：2026-08-18。PRD-088 已完成；下一条权威未完成项为 PRD-089，本次只登记、不实现。总体状态保持 all_108_prds_complete=false。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -5988,16 +5989,244 @@
       <c r="M19" s="21" t="n"/>
       <c r="N19" s="22" t="n"/>
     </row>
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>PRD-088</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>M2-企业增强</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>扩展层</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>白标配置</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>客户/渠道白标配置</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>81/0081 -&gt; 81/0081 -&gt; 80/0080 -&gt; 81/0081；四阶段 integrity=ok、FK=0</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Branding 4/4；Migration 9/9；Console Branding 9/9；Console 全量 935/935；Ruff/lint 通过；真实 HTTP、动态撤权和三视口 Browser 通过</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>docs/testing/PRD-088-tests.md#3-migration-与数据库</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>docs/testing/PRD-088-tests.md#5-browser-page-120</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-088-tenant-white-label-branding.md；docs/api/branding.md；docs/testing/PRD-088-tests.md</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>PRD-088 权威证据摘要</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Runtime SQLite</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>81/0081；integrity_check=ok；外键违规0；Branding audit/event/outbox=3/3/3；outbox pending=0；敏感哨兵=0</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="21" t="n"/>
+      <c r="G22" s="21" t="n"/>
+      <c r="H22" s="21" t="n"/>
+      <c r="I22" s="21" t="n"/>
+      <c r="J22" s="21" t="n"/>
+      <c r="K22" s="21" t="n"/>
+      <c r="L22" s="21" t="n"/>
+      <c r="M22" s="21" t="n"/>
+      <c r="N22" s="22" t="n"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>HTTP 与 Browser</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>admin/viewer/动态撤权/public fallback/no-store 通过；1280x720、390x844、1440x900 非空、无遮挡、零横向溢出</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="21" t="n"/>
+      <c r="I23" s="21" t="n"/>
+      <c r="J23" s="21" t="n"/>
+      <c r="K23" s="21" t="n"/>
+      <c r="L23" s="21" t="n"/>
+      <c r="M23" s="21" t="n"/>
+      <c r="N23" s="22" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>自动化门禁</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Branding 4/4；Migration 9/9；Console Branding 9/9；Console 全量 935/935；Ruff/lint 通过</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="21" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="21" t="n"/>
+      <c r="M24" s="21" t="n"/>
+      <c r="N24" s="22" t="n"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>自审结论</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>两轮编码前自审闭环；tenant/RBAC、PNG/域名、CAS、审计/EVT-100/outbox、迟到响应和品牌生命周期均通过，无未关闭 P0/P1。</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="21" t="n"/>
+      <c r="F25" s="21" t="n"/>
+      <c r="G25" s="21" t="n"/>
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="21" t="n"/>
+      <c r="J25" s="21" t="n"/>
+      <c r="K25" s="21" t="n"/>
+      <c r="L25" s="21" t="n"/>
+      <c r="M25" s="21" t="n"/>
+      <c r="N25" s="22" t="n"/>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>下一项依据</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Excel 总表第90行、M2/M3第26行、PAGE-121、API-402..406、OBJ-122/123、EVT-101/102、TC-0177/0178 共同确认 PRD-089；本次不实现。</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="21" t="n"/>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="21" t="n"/>
+      <c r="J26" s="21" t="n"/>
+      <c r="K26" s="21" t="n"/>
+      <c r="L26" s="21" t="n"/>
+      <c r="M26" s="21" t="n"/>
+      <c r="N26" s="22" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>总体状态</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>all_108_prds_complete=false</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="21" t="n"/>
+      <c r="G27" s="21" t="n"/>
+      <c r="H27" s="21" t="n"/>
+      <c r="I27" s="21" t="n"/>
+      <c r="J27" s="21" t="n"/>
+      <c r="K27" s="21" t="n"/>
+      <c r="L27" s="21" t="n"/>
+      <c r="M27" s="21" t="n"/>
+      <c r="N27" s="22" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A4:N12"/>
-  <mergeCells count="9">
+  <mergeCells count="16">
+    <mergeCell ref="B22:N22"/>
+    <mergeCell ref="B14:N14"/>
     <mergeCell ref="A13:N13"/>
-    <mergeCell ref="B14:N14"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="B27:N27"/>
+    <mergeCell ref="A21:N21"/>
     <mergeCell ref="A2:N2"/>
+    <mergeCell ref="B17:N17"/>
     <mergeCell ref="B18:N18"/>
-    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="B26:N26"/>
     <mergeCell ref="B19:N19"/>
     <mergeCell ref="B15:N15"/>
+    <mergeCell ref="B25:N25"/>
+    <mergeCell ref="B24:N24"/>
     <mergeCell ref="B16:N16"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: complete PRD-089 tenant data export deletion
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5201,11 +5201,10 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>更新时间：2026-08-18。PRD-088 已完成；下一条权威未完成项为 PRD-089，本次只登记、不实现。总体状态保持 all_108_prds_complete=false。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Updated 2026-08-18: PRD-089 completed; PRD-090 is the next unfinished item; all_108_prds_complete=false.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -6122,7 +6121,7 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Branding 4/4；Migration 9/9；Console Branding 9/9；Console 全量 935/935；Ruff/lint 通过</t>
+          <t>PRD-089 final gate: backend 6 passed; migration 0082 fresh/round-trip passed; browser desktop/mobile passed; Console 6 passed; lint 296 files; Control health and ready 200.</t>
         </is>
       </c>
       <c r="C24" s="21" t="n"/>
@@ -6146,7 +6145,7 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>两轮编码前自审闭环；tenant/RBAC、PNG/域名、CAS、审计/EVT-100/outbox、迟到响应和品牌生命周期均通过，无未关闭 P0/P1。</t>
+          <t>Tenant isolation, backend RBAC, export encryption/download integrity, deletion retention, webhook summaries, privacy audit, and no open P0/P1 passed.</t>
         </is>
       </c>
       <c r="C25" s="21" t="n"/>
@@ -6170,7 +6169,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Excel 总表第90行、M2/M3第26行、PAGE-121、API-402..406、OBJ-122/123、EVT-101/102、TC-0177/0178 共同确认 PRD-089；本次不实现。</t>
+          <t>Cross-checked next unfinished item: PRD-090. It is not coded, tested, migrated, or marked complete.</t>
         </is>
       </c>
       <c r="C26" s="21" t="n"/>

</xml_diff>

<commit_message>
docs: complete PRD-090 SaaS architecture baseline
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
+++ b/企业级AI_Gateway_PRD开发总清单_给CodexClaude.xlsx
@@ -5201,7 +5201,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Updated 2026-08-18: PRD-089 completed; PRD-090 is the next unfinished item; all_108_prds_complete=false.</t>
+          <t>Updated 2026-08-20: PRD-001..089 completed; legacy PRD-090..108 retired and forbidden; all_108_prds_complete=false.</t>
         </is>
       </c>
     </row>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Cross-checked next unfinished item: PRD-090. It is not coded, tested, migrated, or marked complete.</t>
+          <t>Legacy PRD-090..108 are retained only for audit and are not active work. The next item is defined only by 企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx; all_108_prds_complete=false.</t>
         </is>
       </c>
       <c r="C26" s="21" t="n"/>

</xml_diff>